<commit_message>
Sprint 19 Code Merged
</commit_message>
<xml_diff>
--- a/reports/bugs/missing-testid-locations.xlsx
+++ b/reports/bugs/missing-testid-locations.xlsx
@@ -8,7 +8,7 @@
     <sheet name="How to locate" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Missing testids'!A1:P106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Missing testids'!A1:P112</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -419,7 +419,7 @@
         <v>What this is</v>
       </c>
       <c r="B3" t="str">
-        <v>105 interactive elements in Setup &gt; Location Settings that have no data-testid of their own.</v>
+        <v>111 interactive elements in Setup &gt; Location Settings that have no data-testid of their own.</v>
       </c>
     </row>
     <row r="4">
@@ -443,7 +443,7 @@
         <v>Report date</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-09-17</v>
+        <v>2026-09-28</v>
       </c>
     </row>
     <row r="7">
@@ -527,12 +527,12 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Child — 24 of the 105 elements sit inside a container that already carries a data-testid. Only the element itself is missing one, and a single attribute closes the gap.</v>
+        <v>Child — 27 of the 111 elements sit inside a container that already carries a data-testid. Only the element itself is missing one, and a single attribute closes the gap.</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Parent and child — the other 81 have no data-testid anywhere in their path. The container needs one too, or the new attribute is still only reachable by text or by counting rows.</v>
+        <v>Parent and child — the other 84 have no data-testid anywhere in their path. The container needs one too, or the new attribute is still only reachable by text or by counting rows.</v>
       </c>
     </row>
     <row r="22">
@@ -581,7 +581,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="B27">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C27" t="str">
         <v>Found by placeholder, form name, aria-label or a CSS class — stable today, implicit and easy to break</v>
@@ -592,7 +592,7 @@
         <v>LOW</v>
       </c>
       <c r="B28">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C28" t="str">
         <v>Inside a container that has a testid — works today, would be more robust with its own</v>
@@ -651,7 +651,7 @@
         <v>Shared dialogs (all Location Settings tabs)</v>
       </c>
       <c r="B36">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="37">
@@ -680,18 +680,18 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Currency tab</v>
+        <v>Location Management History tab</v>
       </c>
       <c r="B40">
-        <v>3</v>
+        <v>14</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Location Management History tab</v>
+        <v>Currency tab</v>
       </c>
       <c r="B41">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="43">
@@ -851,7 +851,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P106"/>
+  <dimension ref="A1:P112"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -5193,10 +5193,10 @@
         <v>Location Management History</v>
       </c>
       <c r="D81" t="str">
-        <v>set Rows Per Page dropdown option</v>
+        <v>Current page number input field</v>
       </c>
       <c r="E81" t="str">
-        <v>[role="option"]</v>
+        <v>[data-testid="location-settings-tab-content-management-history"] input[aria-label="Current page number"]</v>
       </c>
       <c r="F81" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
@@ -5205,28 +5205,28 @@
 4. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
       </c>
       <c r="G81" t="str">
-        <v>Parent and child</v>
+        <v>Child</v>
       </c>
       <c r="H81" t="str">
-        <v>Nothing in the path has a data-testid — the element needs one AND so does the container it sits in (the dialog, table or section), or the element stays reachable only by text or position.</v>
+        <v>Child element only — the container "location-settings-tab-content-management-history" already has a data-testid; add one to the element inside it.</v>
       </c>
       <c r="I81" t="str">
         <v>MEDIUM</v>
       </c>
       <c r="J81" t="str">
-        <v>location-settings-option-management-history</v>
+        <v>location-settings-input-current-page-number</v>
       </c>
       <c r="K81" t="str">
-        <v>none</v>
+        <v>location-settings-tab-content-management-history</v>
       </c>
       <c r="L81" t="str">
-        <v>[role="option"]</v>
+        <v>[data-testid="location-settings-tab-content-management-history"] input[aria-label="Current page number"]</v>
       </c>
       <c r="M81" t="str">
         <v/>
       </c>
       <c r="N81" t="str">
-        <v>$$('[role="option"]')</v>
+        <v>$$('[data-testid="location-settings-tab-content-management-history"] input[aria-label="Current page number"]')</v>
       </c>
       <c r="O81" t="str">
         <v/>
@@ -5246,10 +5246,10 @@
         <v>Location Management History</v>
       </c>
       <c r="D82" t="str">
-        <v>Current page number input field</v>
+        <v>is Read Only tab panel</v>
       </c>
       <c r="E82" t="str">
-        <v>[data-testid="location-settings-tab-content-management-history"] input[aria-label="Current page number"]</v>
+        <v>[role="tabpanel"]</v>
       </c>
       <c r="F82" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
@@ -5258,28 +5258,28 @@
 4. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
       </c>
       <c r="G82" t="str">
-        <v>Child</v>
+        <v>Parent and child</v>
       </c>
       <c r="H82" t="str">
-        <v>Child element only — the container "location-settings-tab-content-management-history" already has a data-testid; add one to the element inside it.</v>
+        <v>Nothing in the path has a data-testid — the element needs one AND so does the container it sits in (the dialog, table or section), or the element stays reachable only by text or position.</v>
       </c>
       <c r="I82" t="str">
         <v>MEDIUM</v>
       </c>
       <c r="J82" t="str">
-        <v>location-settings-input-current-page-number</v>
+        <v>location-settings-sub-tab-content-management-history</v>
       </c>
       <c r="K82" t="str">
-        <v>location-settings-tab-content-management-history</v>
+        <v>none</v>
       </c>
       <c r="L82" t="str">
-        <v>[data-testid="location-settings-tab-content-management-history"] input[aria-label="Current page number"]</v>
+        <v>[role="tabpanel"]</v>
       </c>
       <c r="M82" t="str">
         <v/>
       </c>
       <c r="N82" t="str">
-        <v>$$('[data-testid="location-settings-tab-content-management-history"] input[aria-label="Current page number"]')</v>
+        <v>$$('[role="tabpanel"]')</v>
       </c>
       <c r="O82" t="str">
         <v/>
@@ -5299,10 +5299,10 @@
         <v>Location Management History</v>
       </c>
       <c r="D83" t="str">
-        <v>is Read Only tab panel</v>
+        <v>open Settings Tab tab</v>
       </c>
       <c r="E83" t="str">
-        <v>[role="tabpanel"]</v>
+        <v>[role="tab"]</v>
       </c>
       <c r="F83" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
@@ -5320,19 +5320,19 @@
         <v>MEDIUM</v>
       </c>
       <c r="J83" t="str">
-        <v>location-settings-sub-tab-content-management-history</v>
+        <v>location-settings-sub-tab-management-history</v>
       </c>
       <c r="K83" t="str">
         <v>none</v>
       </c>
       <c r="L83" t="str">
-        <v>[role="tabpanel"]</v>
+        <v>[role="tab"]</v>
       </c>
       <c r="M83" t="str">
         <v/>
       </c>
       <c r="N83" t="str">
-        <v>$$('[role="tabpanel"]')</v>
+        <v>$$('[role="tab"]')</v>
       </c>
       <c r="O83" t="str">
         <v/>
@@ -5352,10 +5352,10 @@
         <v>Location Management History</v>
       </c>
       <c r="D84" t="str">
-        <v>Mgmt History Rows Per Page dropdown</v>
+        <v>write Setting dropdown option</v>
       </c>
       <c r="E84" t="str">
-        <v>[data-testid="location-settings-tab-content-management-history"] button[role="combobox"]:not([data-testid="location-settings-select-history-type"])</v>
+        <v>[role="option"]</v>
       </c>
       <c r="F84" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
@@ -5364,28 +5364,28 @@
 4. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
       </c>
       <c r="G84" t="str">
-        <v>Child</v>
+        <v>Parent and child</v>
       </c>
       <c r="H84" t="str">
-        <v>Child element only — the container "location-settings-tab-content-management-history" already has a data-testid; add one to the element inside it.</v>
+        <v>Nothing in the path has a data-testid — the element needs one AND so does the container it sits in (the dialog, table or section), or the element stays reachable only by text or position.</v>
       </c>
       <c r="I84" t="str">
         <v>MEDIUM</v>
       </c>
       <c r="J84" t="str">
-        <v>location-settings-select-mgmt-history-rows-per-page</v>
+        <v>location-settings-option-management-history</v>
       </c>
       <c r="K84" t="str">
-        <v>location-settings-tab-content-management-history</v>
+        <v>none</v>
       </c>
       <c r="L84" t="str">
-        <v>[data-testid="location-settings-tab-content-management-history"] button[role="combobox"]:not([data-testid="location-settings-select-history-type"])</v>
+        <v>[role="option"]</v>
       </c>
       <c r="M84" t="str">
         <v/>
       </c>
       <c r="N84" t="str">
-        <v>$$('[data-testid="location-settings-tab-content-management-history"] button[role="combobox"]:not([data-testid="location-settings-select-history-type"])')</v>
+        <v>$$('[role="option"]')</v>
       </c>
       <c r="O84" t="str">
         <v/>
@@ -5405,10 +5405,10 @@
         <v>Location Management History</v>
       </c>
       <c r="D85" t="str">
-        <v>Mgmt History First Page button</v>
+        <v>Mgmt History Rows Per Page dropdown</v>
       </c>
       <c r="E85" t="str">
-        <v>button[aria-label="Go to first page"]</v>
+        <v>[data-testid="location-settings-tab-content-management-history"] button[role="combobox"]:not([data-testid="location-settings-select-history-type"])</v>
       </c>
       <c r="F85" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
@@ -5417,28 +5417,28 @@
 4. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
       </c>
       <c r="G85" t="str">
-        <v>Parent and child</v>
+        <v>Child</v>
       </c>
       <c r="H85" t="str">
-        <v>Nothing in the path has a data-testid — the element needs one AND so does the container it sits in (the dialog, table or section), or the element stays reachable only by text or position.</v>
+        <v>Child element only — the container "location-settings-tab-content-management-history" already has a data-testid; add one to the element inside it.</v>
       </c>
       <c r="I85" t="str">
         <v>MEDIUM</v>
       </c>
       <c r="J85" t="str">
-        <v>location-settings-btn-mgmt-history-first-page</v>
+        <v>location-settings-select-mgmt-history-rows-per-page</v>
       </c>
       <c r="K85" t="str">
-        <v>none</v>
+        <v>location-settings-tab-content-management-history</v>
       </c>
       <c r="L85" t="str">
-        <v>button[aria-label="Go to first page"]</v>
+        <v>[data-testid="location-settings-tab-content-management-history"] button[role="combobox"]:not([data-testid="location-settings-select-history-type"])</v>
       </c>
       <c r="M85" t="str">
         <v/>
       </c>
       <c r="N85" t="str">
-        <v>$$('button[aria-label="Go to first page"]')</v>
+        <v>$$('[data-testid="location-settings-tab-content-management-history"] button[role="combobox"]:not([data-testid="location-settings-select-history-type"])')</v>
       </c>
       <c r="O85" t="str">
         <v/>
@@ -5458,10 +5458,10 @@
         <v>Location Management History</v>
       </c>
       <c r="D86" t="str">
-        <v>Mgmt History Prev Page button</v>
+        <v>Mgmt History Current Page input field</v>
       </c>
       <c r="E86" t="str">
-        <v>button[aria-label="Go to previous page"]</v>
+        <v>[data-testid="location-settings-tab-content-management-history"] input[aria-label="Current page number"]</v>
       </c>
       <c r="F86" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
@@ -5470,28 +5470,28 @@
 4. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
       </c>
       <c r="G86" t="str">
-        <v>Parent and child</v>
+        <v>Child</v>
       </c>
       <c r="H86" t="str">
-        <v>Nothing in the path has a data-testid — the element needs one AND so does the container it sits in (the dialog, table or section), or the element stays reachable only by text or position.</v>
+        <v>Child element only — the container "location-settings-tab-content-management-history" already has a data-testid; add one to the element inside it.</v>
       </c>
       <c r="I86" t="str">
         <v>MEDIUM</v>
       </c>
       <c r="J86" t="str">
-        <v>location-settings-btn-mgmt-history-prev-page</v>
+        <v>location-settings-input-mgmt-history-current-page</v>
       </c>
       <c r="K86" t="str">
-        <v>none</v>
+        <v>location-settings-tab-content-management-history</v>
       </c>
       <c r="L86" t="str">
-        <v>button[aria-label="Go to previous page"]</v>
+        <v>[data-testid="location-settings-tab-content-management-history"] input[aria-label="Current page number"]</v>
       </c>
       <c r="M86" t="str">
         <v/>
       </c>
       <c r="N86" t="str">
-        <v>$$('button[aria-label="Go to previous page"]')</v>
+        <v>$$('[data-testid="location-settings-tab-content-management-history"] input[aria-label="Current page number"]')</v>
       </c>
       <c r="O86" t="str">
         <v/>
@@ -5511,10 +5511,10 @@
         <v>Location Management History</v>
       </c>
       <c r="D87" t="str">
-        <v>Mgmt History Next Page button</v>
+        <v>Mgmt History First Page button</v>
       </c>
       <c r="E87" t="str">
-        <v>button[aria-label="Go to next page"]</v>
+        <v>button[aria-label="Go to first page"]</v>
       </c>
       <c r="F87" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
@@ -5532,19 +5532,19 @@
         <v>MEDIUM</v>
       </c>
       <c r="J87" t="str">
-        <v>location-settings-btn-mgmt-history-next-page</v>
+        <v>location-settings-btn-mgmt-history-first-page</v>
       </c>
       <c r="K87" t="str">
         <v>none</v>
       </c>
       <c r="L87" t="str">
-        <v>button[aria-label="Go to next page"]</v>
+        <v>button[aria-label="Go to first page"]</v>
       </c>
       <c r="M87" t="str">
         <v/>
       </c>
       <c r="N87" t="str">
-        <v>$$('button[aria-label="Go to next page"]')</v>
+        <v>$$('button[aria-label="Go to first page"]')</v>
       </c>
       <c r="O87" t="str">
         <v/>
@@ -5564,10 +5564,10 @@
         <v>Location Management History</v>
       </c>
       <c r="D88" t="str">
-        <v>Mgmt History Last Page button</v>
+        <v>Mgmt History Prev Page button</v>
       </c>
       <c r="E88" t="str">
-        <v>button[aria-label="Go to last page"]</v>
+        <v>button[aria-label="Go to previous page"]</v>
       </c>
       <c r="F88" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
@@ -5585,19 +5585,19 @@
         <v>MEDIUM</v>
       </c>
       <c r="J88" t="str">
-        <v>location-settings-btn-mgmt-history-last-page</v>
+        <v>location-settings-btn-mgmt-history-prev-page</v>
       </c>
       <c r="K88" t="str">
         <v>none</v>
       </c>
       <c r="L88" t="str">
-        <v>button[aria-label="Go to last page"]</v>
+        <v>button[aria-label="Go to previous page"]</v>
       </c>
       <c r="M88" t="str">
         <v/>
       </c>
       <c r="N88" t="str">
-        <v>$$('button[aria-label="Go to last page"]')</v>
+        <v>$$('button[aria-label="Go to previous page"]')</v>
       </c>
       <c r="O88" t="str">
         <v/>
@@ -5608,978 +5608,1297 @@
     </row>
     <row r="89" xml:space="preserve">
       <c r="A89" t="str">
+        <v>HIS-011</v>
+      </c>
+      <c r="B89" t="str">
+        <v>Location Settings</v>
+      </c>
+      <c r="C89" t="str">
+        <v>Location Management History</v>
+      </c>
+      <c r="D89" t="str">
+        <v>Mgmt History Next Page button</v>
+      </c>
+      <c r="E89" t="str">
+        <v>button[aria-label="Go to next page"]</v>
+      </c>
+      <c r="F89" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Sign in to Navigator Cloud.
+2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
+3. Open the Location Management History tab.
+4. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
+      </c>
+      <c r="G89" t="str">
+        <v>Parent and child</v>
+      </c>
+      <c r="H89" t="str">
+        <v>Nothing in the path has a data-testid — the element needs one AND so does the container it sits in (the dialog, table or section), or the element stays reachable only by text or position.</v>
+      </c>
+      <c r="I89" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="J89" t="str">
+        <v>location-settings-btn-mgmt-history-next-page</v>
+      </c>
+      <c r="K89" t="str">
+        <v>none</v>
+      </c>
+      <c r="L89" t="str">
+        <v>button[aria-label="Go to next page"]</v>
+      </c>
+      <c r="M89" t="str">
+        <v/>
+      </c>
+      <c r="N89" t="str">
+        <v>$$('button[aria-label="Go to next page"]')</v>
+      </c>
+      <c r="O89" t="str">
+        <v/>
+      </c>
+      <c r="P89" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="90" xml:space="preserve">
+      <c r="A90" t="str">
+        <v>HIS-012</v>
+      </c>
+      <c r="B90" t="str">
+        <v>Location Settings</v>
+      </c>
+      <c r="C90" t="str">
+        <v>Location Management History</v>
+      </c>
+      <c r="D90" t="str">
+        <v>Mgmt History Last Page button</v>
+      </c>
+      <c r="E90" t="str">
+        <v>button[aria-label="Go to last page"]</v>
+      </c>
+      <c r="F90" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Sign in to Navigator Cloud.
+2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
+3. Open the Location Management History tab.
+4. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
+      </c>
+      <c r="G90" t="str">
+        <v>Parent and child</v>
+      </c>
+      <c r="H90" t="str">
+        <v>Nothing in the path has a data-testid — the element needs one AND so does the container it sits in (the dialog, table or section), or the element stays reachable only by text or position.</v>
+      </c>
+      <c r="I90" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="J90" t="str">
+        <v>location-settings-btn-mgmt-history-last-page</v>
+      </c>
+      <c r="K90" t="str">
+        <v>none</v>
+      </c>
+      <c r="L90" t="str">
+        <v>button[aria-label="Go to last page"]</v>
+      </c>
+      <c r="M90" t="str">
+        <v/>
+      </c>
+      <c r="N90" t="str">
+        <v>$$('button[aria-label="Go to last page"]')</v>
+      </c>
+      <c r="O90" t="str">
+        <v/>
+      </c>
+      <c r="P90" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="91" xml:space="preserve">
+      <c r="A91" t="str">
         <v>NOT-003</v>
       </c>
-      <c r="B89" t="str">
-        <v>Location Settings</v>
-      </c>
-      <c r="C89" t="str">
+      <c r="B91" t="str">
+        <v>Location Settings</v>
+      </c>
+      <c r="C91" t="str">
         <v>Notes</v>
       </c>
-      <c r="D89" t="str">
+      <c r="D91" t="str">
         <v>Note Row0 input field</v>
       </c>
-      <c r="E89" t="str">
+      <c r="E91" t="str">
         <v>textarea[name="notes.notes.0.note"]</v>
       </c>
-      <c r="F89" t="str" xml:space="preserve">
+      <c r="F91" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
 2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
 3. Open the Notes tab.
 4. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
       </c>
-      <c r="G89" t="str">
-        <v>Parent and child</v>
-      </c>
-      <c r="H89" t="str">
-        <v>Nothing in the path has a data-testid — the element needs one AND so does the container it sits in (the dialog, table or section), or the element stays reachable only by text or position.</v>
-      </c>
-      <c r="I89" t="str">
+      <c r="G91" t="str">
+        <v>Parent and child</v>
+      </c>
+      <c r="H91" t="str">
+        <v>Nothing in the path has a data-testid — the element needs one AND so does the container it sits in (the dialog, table or section), or the element stays reachable only by text or position.</v>
+      </c>
+      <c r="I91" t="str">
         <v>MEDIUM</v>
       </c>
-      <c r="J89" t="str">
+      <c r="J91" t="str">
         <v>location-settings-input-note-row-0</v>
       </c>
-      <c r="K89" t="str">
-        <v>none</v>
-      </c>
-      <c r="L89" t="str">
+      <c r="K91" t="str">
+        <v>none</v>
+      </c>
+      <c r="L91" t="str">
         <v>textarea[name="notes.notes.0.note"]</v>
       </c>
-      <c r="M89" t="str">
-        <v/>
-      </c>
-      <c r="N89" t="str">
+      <c r="M91" t="str">
+        <v/>
+      </c>
+      <c r="N91" t="str">
         <v>$$('textarea[name="notes.notes.0.note"]')</v>
       </c>
-      <c r="O89" t="str">
-        <v/>
-      </c>
-      <c r="P89" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="90" xml:space="preserve">
-      <c r="A90" t="str">
+      <c r="O91" t="str">
+        <v/>
+      </c>
+      <c r="P91" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="92" xml:space="preserve">
+      <c r="A92" t="str">
         <v>PRI-011</v>
       </c>
-      <c r="B90" t="str">
-        <v>Location Settings</v>
-      </c>
-      <c r="C90" t="str">
+      <c r="B92" t="str">
+        <v>Location Settings</v>
+      </c>
+      <c r="C92" t="str">
         <v>Pricing</v>
       </c>
-      <c r="D90" t="str">
+      <c r="D92" t="str">
         <v>select Date From Calendar cell</v>
       </c>
-      <c r="E90" t="str">
+      <c r="E92" t="str">
         <v>[role="gridcell"]</v>
       </c>
-      <c r="F90" t="str" xml:space="preserve">
+      <c r="F92" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
 2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
 3. Open the Pricing tab.
 4. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
       </c>
-      <c r="G90" t="str">
-        <v>Parent and child</v>
-      </c>
-      <c r="H90" t="str">
-        <v>Nothing in the path has a data-testid — the element needs one AND so does the container it sits in (the dialog, table or section), or the element stays reachable only by text or position.</v>
-      </c>
-      <c r="I90" t="str">
+      <c r="G92" t="str">
+        <v>Parent and child</v>
+      </c>
+      <c r="H92" t="str">
+        <v>Nothing in the path has a data-testid — the element needs one AND so does the container it sits in (the dialog, table or section), or the element stays reachable only by text or position.</v>
+      </c>
+      <c r="I92" t="str">
         <v>MEDIUM</v>
       </c>
-      <c r="J90" t="str">
+      <c r="J92" t="str">
         <v>location-settings-cell-pricing</v>
       </c>
-      <c r="K90" t="str">
-        <v>none</v>
-      </c>
-      <c r="L90" t="str">
+      <c r="K92" t="str">
+        <v>none</v>
+      </c>
+      <c r="L92" t="str">
         <v>[role="gridcell"]</v>
       </c>
-      <c r="M90" t="str">
-        <v/>
-      </c>
-      <c r="N90" t="str">
+      <c r="M92" t="str">
+        <v/>
+      </c>
+      <c r="N92" t="str">
         <v>$$('[role="gridcell"]')</v>
       </c>
-      <c r="O90" t="str">
-        <v/>
-      </c>
-      <c r="P90" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="91" xml:space="preserve">
-      <c r="A91" t="str">
+      <c r="O92" t="str">
+        <v/>
+      </c>
+      <c r="P92" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="93" xml:space="preserve">
+      <c r="A93" t="str">
         <v>PRI-012</v>
       </c>
-      <c r="B91" t="str">
-        <v>Location Settings</v>
-      </c>
-      <c r="C91" t="str">
+      <c r="B93" t="str">
+        <v>Location Settings</v>
+      </c>
+      <c r="C93" t="str">
         <v>Pricing</v>
       </c>
-      <c r="D91" t="str">
+      <c r="D93" t="str">
         <v>select Date From Calendar button</v>
       </c>
-      <c r="E91" t="str">
+      <c r="E93" t="str">
         <v>[role="button"]</v>
       </c>
-      <c r="F91" t="str" xml:space="preserve">
+      <c r="F93" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
 2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
 3. Open the Pricing tab.
 4. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
       </c>
-      <c r="G91" t="str">
-        <v>Parent and child</v>
-      </c>
-      <c r="H91" t="str">
-        <v>Nothing in the path has a data-testid — the element needs one AND so does the container it sits in (the dialog, table or section), or the element stays reachable only by text or position.</v>
-      </c>
-      <c r="I91" t="str">
+      <c r="G93" t="str">
+        <v>Parent and child</v>
+      </c>
+      <c r="H93" t="str">
+        <v>Nothing in the path has a data-testid — the element needs one AND so does the container it sits in (the dialog, table or section), or the element stays reachable only by text or position.</v>
+      </c>
+      <c r="I93" t="str">
         <v>MEDIUM</v>
       </c>
-      <c r="J91" t="str">
+      <c r="J93" t="str">
         <v>location-settings-btn-pricing</v>
       </c>
-      <c r="K91" t="str">
-        <v>none</v>
-      </c>
-      <c r="L91" t="str">
+      <c r="K93" t="str">
+        <v>none</v>
+      </c>
+      <c r="L93" t="str">
         <v>[role="button"]</v>
       </c>
-      <c r="M91" t="str">
-        <v/>
-      </c>
-      <c r="N91" t="str">
+      <c r="M93" t="str">
+        <v/>
+      </c>
+      <c r="N93" t="str">
         <v>$$('[role="button"]')</v>
       </c>
-      <c r="O91" t="str">
-        <v/>
-      </c>
-      <c r="P91" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="92" xml:space="preserve">
-      <c r="A92" t="str">
+      <c r="O93" t="str">
+        <v/>
+      </c>
+      <c r="P93" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="94" xml:space="preserve">
+      <c r="A94" t="str">
+        <v>DLG-007</v>
+      </c>
+      <c r="B94" t="str">
+        <v>Location Settings</v>
+      </c>
+      <c r="C94" t="str">
+        <v>Shared dialogs (all tabs)</v>
+      </c>
+      <c r="D94" t="str">
+        <v>User Menu button</v>
+      </c>
+      <c r="E94" t="str">
+        <v>[data-sidebar="footer"] button[data-slot="dropdown-menu-trigger"]</v>
+      </c>
+      <c r="F94" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Sign in to Navigator Cloud.
+2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
+3. Open any tab — this surface is shared by all of them.
+4. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
+      </c>
+      <c r="G94" t="str">
+        <v>Parent and child</v>
+      </c>
+      <c r="H94" t="str">
+        <v>Nothing in the path has a data-testid — the element needs one AND so does the container it sits in (the dialog, table or section), or the element stays reachable only by text or position.</v>
+      </c>
+      <c r="I94" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="J94" t="str">
+        <v>location-settings-btn-user-menu</v>
+      </c>
+      <c r="K94" t="str">
+        <v>none</v>
+      </c>
+      <c r="L94" t="str">
+        <v>[data-sidebar="footer"] button[data-slot="dropdown-menu-trigger"]</v>
+      </c>
+      <c r="M94" t="str">
+        <v/>
+      </c>
+      <c r="N94" t="str">
+        <v>$$('[data-sidebar="footer"] button[data-slot="dropdown-menu-trigger"]')</v>
+      </c>
+      <c r="O94" t="str">
+        <v/>
+      </c>
+      <c r="P94" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="95" xml:space="preserve">
+      <c r="A95" t="str">
+        <v>DLG-008</v>
+      </c>
+      <c r="B95" t="str">
+        <v>Location Settings</v>
+      </c>
+      <c r="C95" t="str">
+        <v>Shared dialogs (all tabs)</v>
+      </c>
+      <c r="D95" t="str">
+        <v>mnu Language element</v>
+      </c>
+      <c r="E95" t="str">
+        <v>[role="menu"] [role="menuitem"][aria-haspopup="menu"]</v>
+      </c>
+      <c r="F95" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Sign in to Navigator Cloud.
+2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
+3. Open any tab — this surface is shared by all of them.
+4. Click a column header, then open its menu.
+5. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
+      </c>
+      <c r="G95" t="str">
+        <v>Parent and child</v>
+      </c>
+      <c r="H95" t="str">
+        <v>Nothing in the path has a data-testid — the element needs one AND so does the container it sits in (the dialog, table or section), or the element stays reachable only by text or position.</v>
+      </c>
+      <c r="I95" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="J95" t="str">
+        <v>location-settings-mnu-language</v>
+      </c>
+      <c r="K95" t="str">
+        <v>none</v>
+      </c>
+      <c r="L95" t="str">
+        <v>[role="menu"] [role="menuitem"][aria-haspopup="menu"]</v>
+      </c>
+      <c r="M95" t="str">
+        <v/>
+      </c>
+      <c r="N95" t="str">
+        <v>$$('[role="menu"] [role="menuitem"][aria-haspopup="menu"]')</v>
+      </c>
+      <c r="O95" t="str">
+        <v/>
+      </c>
+      <c r="P95" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="96" xml:space="preserve">
+      <c r="A96" t="str">
         <v>AA-016</v>
       </c>
-      <c r="B92" t="str">
-        <v>Location Settings</v>
-      </c>
-      <c r="C92" t="str">
+      <c r="B96" t="str">
+        <v>Location Settings</v>
+      </c>
+      <c r="C96" t="str">
         <v>Account and Address</v>
       </c>
-      <c r="D92" t="str">
+      <c r="D96" t="str">
         <v>Venue/Branch Account element</v>
       </c>
-      <c r="E92" t="str">
+      <c r="E96" t="str">
         <v>[data-testid="location-settings-sub-tab-content-account-and-address"] :text("Venue/Branch Account")</v>
       </c>
-      <c r="F92" t="str" xml:space="preserve">
+      <c r="F96" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
 2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
 3. Open the Account and Address tab.
 4. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
       </c>
-      <c r="G92" t="str">
+      <c r="G96" t="str">
         <v>Child</v>
       </c>
-      <c r="H92" t="str">
+      <c r="H96" t="str">
         <v>Child element only — the container "location-settings-sub-tab-content-account-and-address" already has a data-testid; add one to the element inside it.</v>
       </c>
-      <c r="I92" t="str">
+      <c r="I96" t="str">
         <v>LOW</v>
       </c>
-      <c r="J92" t="str">
+      <c r="J96" t="str">
         <v>location-settings-venue-branch-account</v>
       </c>
-      <c r="K92" t="str">
+      <c r="K96" t="str">
         <v>location-settings-sub-tab-content-account-and-address</v>
       </c>
-      <c r="L92" t="str">
+      <c r="L96" t="str">
         <v>[data-testid="location-settings-sub-tab-content-account-and-address"]</v>
       </c>
-      <c r="M92" t="str">
+      <c r="M96" t="str">
         <v>Venue/Branch Account</v>
       </c>
-      <c r="N92" t="str">
+      <c r="N96" t="str">
         <v>$$('[data-testid="location-settings-sub-tab-content-account-and-address"]').filter(e =&gt; (e.innerText || e.getAttribute('aria-label') || e.placeholder || '').includes('Venue/Branch Account'))</v>
       </c>
-      <c r="O92" t="str">
-        <v/>
-      </c>
-      <c r="P92" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="93" xml:space="preserve">
-      <c r="A93" t="str">
+      <c r="O96" t="str">
+        <v/>
+      </c>
+      <c r="P96" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="97" xml:space="preserve">
+      <c r="A97" t="str">
         <v>AA-017</v>
       </c>
-      <c r="B93" t="str">
-        <v>Location Settings</v>
-      </c>
-      <c r="C93" t="str">
+      <c r="B97" t="str">
+        <v>Location Settings</v>
+      </c>
+      <c r="C97" t="str">
         <v>Account and Address</v>
       </c>
-      <c r="D93" t="str">
+      <c r="D97" t="str">
         <v>Master Bill To Address element</v>
       </c>
-      <c r="E93" t="str">
+      <c r="E97" t="str">
         <v>[data-testid="location-settings-sub-tab-content-account-and-address"] :text("Master Bill To Address")</v>
       </c>
-      <c r="F93" t="str" xml:space="preserve">
+      <c r="F97" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
 2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
 3. Open the Account and Address tab.
 4. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
       </c>
-      <c r="G93" t="str">
+      <c r="G97" t="str">
         <v>Child</v>
       </c>
-      <c r="H93" t="str">
+      <c r="H97" t="str">
         <v>Child element only — the container "location-settings-sub-tab-content-account-and-address" already has a data-testid; add one to the element inside it.</v>
       </c>
-      <c r="I93" t="str">
+      <c r="I97" t="str">
         <v>LOW</v>
       </c>
-      <c r="J93" t="str">
+      <c r="J97" t="str">
         <v>location-settings-master-bill-to-address</v>
       </c>
-      <c r="K93" t="str">
+      <c r="K97" t="str">
         <v>location-settings-sub-tab-content-account-and-address</v>
       </c>
-      <c r="L93" t="str">
+      <c r="L97" t="str">
         <v>[data-testid="location-settings-sub-tab-content-account-and-address"]</v>
       </c>
-      <c r="M93" t="str">
+      <c r="M97" t="str">
         <v>Master Bill To Address</v>
       </c>
-      <c r="N93" t="str">
+      <c r="N97" t="str">
         <v>$$('[data-testid="location-settings-sub-tab-content-account-and-address"]').filter(e =&gt; (e.innerText || e.getAttribute('aria-label') || e.placeholder || '').includes('Master Bill To Address'))</v>
       </c>
-      <c r="O93" t="str">
-        <v/>
-      </c>
-      <c r="P93" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="94" xml:space="preserve">
-      <c r="A94" t="str">
+      <c r="O97" t="str">
+        <v/>
+      </c>
+      <c r="P97" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="98" xml:space="preserve">
+      <c r="A98" t="str">
         <v>AA-018</v>
       </c>
-      <c r="B94" t="str">
-        <v>Location Settings</v>
-      </c>
-      <c r="C94" t="str">
+      <c r="B98" t="str">
+        <v>Location Settings</v>
+      </c>
+      <c r="C98" t="str">
         <v>Account and Address</v>
       </c>
-      <c r="D94" t="str">
+      <c r="D98" t="str">
         <v>is Display Field Read Only element</v>
       </c>
-      <c r="E94" t="str">
+      <c r="E98" t="str">
         <v>[data-testid="location-settings-sub-tab-content-account-and-address"] :text("${sectionText}")</v>
       </c>
-      <c r="F94" t="str" xml:space="preserve">
+      <c r="F98" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
 2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
 3. Open the Account and Address tab.
 4. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
       </c>
-      <c r="G94" t="str">
+      <c r="G98" t="str">
         <v>Child</v>
       </c>
-      <c r="H94" t="str">
+      <c r="H98" t="str">
         <v>Child element only — the container "location-settings-sub-tab-content-account-and-address" already has a data-testid; add one to the element inside it.</v>
       </c>
-      <c r="I94" t="str">
+      <c r="I98" t="str">
         <v>LOW</v>
       </c>
-      <c r="J94" t="str">
+      <c r="J98" t="str">
         <v>location-settings-account-and-address-{section-text}</v>
       </c>
-      <c r="K94" t="str">
+      <c r="K98" t="str">
         <v>location-settings-sub-tab-content-account-and-address</v>
       </c>
-      <c r="L94" t="str">
+      <c r="L98" t="str">
         <v>[data-testid="location-settings-sub-tab-content-account-and-address"]</v>
       </c>
-      <c r="M94" t="str">
-        <v/>
-      </c>
-      <c r="N94" t="str">
+      <c r="M98" t="str">
+        <v/>
+      </c>
+      <c r="N98" t="str">
         <v>$$('[data-testid="location-settings-sub-tab-content-account-and-address"]')</v>
       </c>
-      <c r="O94" t="str">
-        <v/>
-      </c>
-      <c r="P94" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="95" xml:space="preserve">
-      <c r="A95" t="str">
+      <c r="O98" t="str">
+        <v/>
+      </c>
+      <c r="P98" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="99" xml:space="preserve">
+      <c r="A99" t="str">
         <v>AA-019</v>
       </c>
-      <c r="B95" t="str">
-        <v>Location Settings</v>
-      </c>
-      <c r="C95" t="str">
+      <c r="B99" t="str">
+        <v>Location Settings</v>
+      </c>
+      <c r="C99" t="str">
         <v>Account and Address</v>
       </c>
-      <c r="D95" t="str">
+      <c r="D99" t="str">
         <v>account List Results Contain element</v>
       </c>
-      <c r="E95" t="str">
+      <c r="E99" t="str">
         <v>[data-testid="location-settings-modal-account-list"] table tbody:has-text("${text}")</v>
       </c>
-      <c r="F95" t="str" xml:space="preserve">
+      <c r="F99" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
 2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
 3. Open the Account and Address tab.
 4. Click the lookup button beside the Venue/Branch Account name. (opens the account list dialog)
 5. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
       </c>
-      <c r="G95" t="str">
+      <c r="G99" t="str">
         <v>Child</v>
       </c>
-      <c r="H95" t="str">
+      <c r="H99" t="str">
         <v>Child element only — the container "location-settings-modal-account-list" already has a data-testid; add one to the element inside it.</v>
       </c>
-      <c r="I95" t="str">
+      <c r="I99" t="str">
         <v>LOW</v>
       </c>
-      <c r="J95" t="str">
+      <c r="J99" t="str">
         <v>location-settings-account-list-{text}</v>
       </c>
-      <c r="K95" t="str">
+      <c r="K99" t="str">
         <v>location-settings-modal-account-list</v>
       </c>
-      <c r="L95" t="str">
+      <c r="L99" t="str">
         <v>[data-testid="location-settings-modal-account-list"] table tbody</v>
       </c>
-      <c r="M95" t="str">
-        <v/>
-      </c>
-      <c r="N95" t="str">
+      <c r="M99" t="str">
+        <v/>
+      </c>
+      <c r="N99" t="str">
         <v>$$('[data-testid="location-settings-modal-account-list"] table tbody')</v>
       </c>
-      <c r="O95" t="str">
-        <v/>
-      </c>
-      <c r="P95" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="96" xml:space="preserve">
-      <c r="A96" t="str">
+      <c r="O99" t="str">
+        <v/>
+      </c>
+      <c r="P99" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="100" xml:space="preserve">
+      <c r="A100" t="str">
         <v>AA-020</v>
       </c>
-      <c r="B96" t="str">
-        <v>Location Settings</v>
-      </c>
-      <c r="C96" t="str">
+      <c r="B100" t="str">
+        <v>Location Settings</v>
+      </c>
+      <c r="C100" t="str">
         <v>Account and Address</v>
       </c>
-      <c r="D96" t="str">
+      <c r="D100" t="str">
         <v>Acc List Close button</v>
       </c>
-      <c r="E96" t="str">
+      <c r="E100" t="str">
         <v>[data-testid="location-settings-modal-account-list"] button:has-text("Close")</v>
       </c>
-      <c r="F96" t="str" xml:space="preserve">
+      <c r="F100" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
 2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
 3. Open the Account and Address tab.
 4. Click the lookup button beside the Venue/Branch Account name. (opens the account list dialog)
 5. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
       </c>
-      <c r="G96" t="str">
+      <c r="G100" t="str">
         <v>Child</v>
       </c>
-      <c r="H96" t="str">
+      <c r="H100" t="str">
         <v>Child element only — the container "location-settings-modal-account-list" already has a data-testid; add one to the element inside it.</v>
       </c>
-      <c r="I96" t="str">
+      <c r="I100" t="str">
         <v>LOW</v>
       </c>
-      <c r="J96" t="str">
+      <c r="J100" t="str">
         <v>location-settings-btn-acc-list-close</v>
       </c>
-      <c r="K96" t="str">
+      <c r="K100" t="str">
         <v>location-settings-modal-account-list</v>
       </c>
-      <c r="L96" t="str">
+      <c r="L100" t="str">
         <v>[data-testid="location-settings-modal-account-list"] button</v>
       </c>
-      <c r="M96" t="str">
+      <c r="M100" t="str">
         <v>Close</v>
       </c>
-      <c r="N96" t="str">
+      <c r="N100" t="str">
         <v>$$('[data-testid="location-settings-modal-account-list"] button').filter(e =&gt; (e.innerText || e.getAttribute('aria-label') || e.placeholder || '').includes('Close'))</v>
       </c>
-      <c r="O96" t="str">
-        <v/>
-      </c>
-      <c r="P96" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="97" xml:space="preserve">
-      <c r="A97" t="str">
+      <c r="O100" t="str">
+        <v/>
+      </c>
+      <c r="P100" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="101" xml:space="preserve">
+      <c r="A101" t="str">
         <v>AA-021</v>
       </c>
-      <c r="B97" t="str">
-        <v>Location Settings</v>
-      </c>
-      <c r="C97" t="str">
+      <c r="B101" t="str">
+        <v>Location Settings</v>
+      </c>
+      <c r="C101" t="str">
         <v>Account and Address</v>
       </c>
-      <c r="D97" t="str">
+      <c r="D101" t="str">
         <v>Acc List Results table</v>
       </c>
-      <c r="E97" t="str">
+      <c r="E101" t="str">
         <v>[data-testid="location-settings-modal-account-list"] table</v>
       </c>
-      <c r="F97" t="str" xml:space="preserve">
+      <c r="F101" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
 2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
 3. Open the Account and Address tab.
 4. Click the lookup button beside the Venue/Branch Account name. (opens the account list dialog)
 5. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
       </c>
-      <c r="G97" t="str">
+      <c r="G101" t="str">
         <v>Child</v>
       </c>
-      <c r="H97" t="str">
+      <c r="H101" t="str">
         <v>Child element only — the container "location-settings-modal-account-list" already has a data-testid; add one to the element inside it.</v>
       </c>
-      <c r="I97" t="str">
+      <c r="I101" t="str">
         <v>LOW</v>
       </c>
-      <c r="J97" t="str">
+      <c r="J101" t="str">
         <v>location-settings-table-acc-list-results</v>
       </c>
-      <c r="K97" t="str">
+      <c r="K101" t="str">
         <v>location-settings-modal-account-list</v>
       </c>
-      <c r="L97" t="str">
+      <c r="L101" t="str">
         <v>[data-testid="location-settings-modal-account-list"] table</v>
       </c>
-      <c r="M97" t="str">
-        <v/>
-      </c>
-      <c r="N97" t="str">
+      <c r="M101" t="str">
+        <v/>
+      </c>
+      <c r="N101" t="str">
         <v>$$('[data-testid="location-settings-modal-account-list"] table')</v>
       </c>
-      <c r="O97" t="str">
-        <v/>
-      </c>
-      <c r="P97" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="98" xml:space="preserve">
-      <c r="A98" t="str">
+      <c r="O101" t="str">
+        <v/>
+      </c>
+      <c r="P101" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="102" xml:space="preserve">
+      <c r="A102" t="str">
         <v>AAO-006</v>
       </c>
-      <c r="B98" t="str">
-        <v>Location Settings</v>
-      </c>
-      <c r="C98" t="str">
+      <c r="B102" t="str">
+        <v>Location Settings</v>
+      </c>
+      <c r="C102" t="str">
         <v>Auto Add-On</v>
       </c>
-      <c r="D98" t="str">
+      <c r="D102" t="str">
         <v>get Unsaved Dialog Heading label</v>
       </c>
-      <c r="E98" t="str">
+      <c r="E102" t="str">
         <v>[data-testid="location-settings-modal-unsaved-changes"] h2</v>
       </c>
-      <c r="F98" t="str" xml:space="preserve">
+      <c r="F102" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
 2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
 3. Open the Auto Add-On tab.
 4. Change any field, then navigate away without saving (for example click Home in the sidebar). (opens the unsaved changes dialog)
 5. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
       </c>
-      <c r="G98" t="str">
+      <c r="G102" t="str">
         <v>Child</v>
       </c>
-      <c r="H98" t="str">
+      <c r="H102" t="str">
         <v>Child element only — the container "location-settings-modal-unsaved-changes" already has a data-testid; add one to the element inside it.</v>
       </c>
-      <c r="I98" t="str">
+      <c r="I102" t="str">
         <v>LOW</v>
       </c>
-      <c r="J98" t="str">
+      <c r="J102" t="str">
         <v>location-settings-label-unsaved-changes</v>
       </c>
-      <c r="K98" t="str">
+      <c r="K102" t="str">
         <v>location-settings-modal-unsaved-changes</v>
       </c>
-      <c r="L98" t="str">
+      <c r="L102" t="str">
         <v>[data-testid="location-settings-modal-unsaved-changes"] h2</v>
       </c>
-      <c r="M98" t="str">
-        <v/>
-      </c>
-      <c r="N98" t="str">
+      <c r="M102" t="str">
+        <v/>
+      </c>
+      <c r="N102" t="str">
         <v>$$('[data-testid="location-settings-modal-unsaved-changes"] h2')</v>
       </c>
-      <c r="O98" t="str">
-        <v/>
-      </c>
-      <c r="P98" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="99" xml:space="preserve">
-      <c r="A99" t="str">
+      <c r="O102" t="str">
+        <v/>
+      </c>
+      <c r="P102" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="103" xml:space="preserve">
+      <c r="A103" t="str">
+        <v>HIS-013</v>
+      </c>
+      <c r="B103" t="str">
+        <v>Location Settings</v>
+      </c>
+      <c r="C103" t="str">
+        <v>Location Management History</v>
+      </c>
+      <c r="D103" t="str">
+        <v>Delete button</v>
+      </c>
+      <c r="E103" t="str">
+        <v>[data-testid="location-settings-section-notes"] button:has-text("Delete")</v>
+      </c>
+      <c r="F103" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Sign in to Navigator Cloud.
+2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
+3. Open the Location Management History tab.
+4. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
+      </c>
+      <c r="G103" t="str">
+        <v>Child</v>
+      </c>
+      <c r="H103" t="str">
+        <v>Child element only — the container "location-settings-section-notes" already has a data-testid; add one to the element inside it.</v>
+      </c>
+      <c r="I103" t="str">
+        <v>LOW</v>
+      </c>
+      <c r="J103" t="str">
+        <v>location-settings-btn-delete</v>
+      </c>
+      <c r="K103" t="str">
+        <v>location-settings-section-notes</v>
+      </c>
+      <c r="L103" t="str">
+        <v>[data-testid="location-settings-section-notes"] button</v>
+      </c>
+      <c r="M103" t="str">
+        <v>Delete</v>
+      </c>
+      <c r="N103" t="str">
+        <v>$$('[data-testid="location-settings-section-notes"] button').filter(e =&gt; (e.innerText || e.getAttribute('aria-label') || e.placeholder || '').includes('Delete'))</v>
+      </c>
+      <c r="O103" t="str">
+        <v/>
+      </c>
+      <c r="P103" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="104" xml:space="preserve">
+      <c r="A104" t="str">
+        <v>HIS-014</v>
+      </c>
+      <c r="B104" t="str">
+        <v>Location Settings</v>
+      </c>
+      <c r="C104" t="str">
+        <v>Location Management History</v>
+      </c>
+      <c r="D104" t="str">
+        <v>Any Mgmt History table</v>
+      </c>
+      <c r="E104" t="str">
+        <v>[data-testid="location-settings-tab-content-management-history"] table[data-slot="table"]</v>
+      </c>
+      <c r="F104" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Sign in to Navigator Cloud.
+2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
+3. Open the Location Management History tab.
+4. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
+      </c>
+      <c r="G104" t="str">
+        <v>Child</v>
+      </c>
+      <c r="H104" t="str">
+        <v>Child element only — the container "location-settings-tab-content-management-history" already has a data-testid; add one to the element inside it.</v>
+      </c>
+      <c r="I104" t="str">
+        <v>LOW</v>
+      </c>
+      <c r="J104" t="str">
+        <v>location-settings-table-any-mgmt-history</v>
+      </c>
+      <c r="K104" t="str">
+        <v>location-settings-tab-content-management-history</v>
+      </c>
+      <c r="L104" t="str">
+        <v>[data-testid="location-settings-tab-content-management-history"] table[data-slot="table"]</v>
+      </c>
+      <c r="M104" t="str">
+        <v/>
+      </c>
+      <c r="N104" t="str">
+        <v>$$('[data-testid="location-settings-tab-content-management-history"] table[data-slot="table"]')</v>
+      </c>
+      <c r="O104" t="str">
+        <v/>
+      </c>
+      <c r="P104" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="105" xml:space="preserve">
+      <c r="A105" t="str">
         <v>NOT-004</v>
       </c>
-      <c r="B99" t="str">
-        <v>Location Settings</v>
-      </c>
-      <c r="C99" t="str">
+      <c r="B105" t="str">
+        <v>Location Settings</v>
+      </c>
+      <c r="C105" t="str">
         <v>Notes</v>
       </c>
-      <c r="D99" t="str">
+      <c r="D105" t="str">
         <v>Label ("No Notes Available")</v>
       </c>
-      <c r="E99" t="str">
+      <c r="E105" t="str">
         <v>[data-testid="location-settings-section-notes"] td:has-text("No Notes Available")</v>
       </c>
-      <c r="F99" t="str" xml:space="preserve">
+      <c r="F105" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
 2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
 3. Open the Notes tab.
 4. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
       </c>
-      <c r="G99" t="str">
+      <c r="G105" t="str">
         <v>Child</v>
       </c>
-      <c r="H99" t="str">
+      <c r="H105" t="str">
         <v>Child element only — the container "location-settings-section-notes" already has a data-testid; add one to the element inside it.</v>
       </c>
-      <c r="I99" t="str">
+      <c r="I105" t="str">
         <v>LOW</v>
       </c>
-      <c r="J99" t="str">
+      <c r="J105" t="str">
         <v>location-settings-label-no-notes-available</v>
       </c>
-      <c r="K99" t="str">
+      <c r="K105" t="str">
         <v>location-settings-section-notes</v>
       </c>
-      <c r="L99" t="str">
+      <c r="L105" t="str">
         <v>[data-testid="location-settings-section-notes"] td</v>
       </c>
-      <c r="M99" t="str">
+      <c r="M105" t="str">
         <v>No Notes Available</v>
       </c>
-      <c r="N99" t="str">
+      <c r="N105" t="str">
         <v>$$('[data-testid="location-settings-section-notes"] td').filter(e =&gt; (e.innerText || e.getAttribute('aria-label') || e.placeholder || '').includes('No Notes Available'))</v>
       </c>
-      <c r="O99" t="str">
-        <v/>
-      </c>
-      <c r="P99" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="100" xml:space="preserve">
-      <c r="A100" t="str">
+      <c r="O105" t="str">
+        <v/>
+      </c>
+      <c r="P105" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="106" xml:space="preserve">
+      <c r="A106" t="str">
         <v>NOT-005</v>
       </c>
-      <c r="B100" t="str">
-        <v>Location Settings</v>
-      </c>
-      <c r="C100" t="str">
+      <c r="B106" t="str">
+        <v>Location Settings</v>
+      </c>
+      <c r="C106" t="str">
         <v>Notes</v>
       </c>
-      <c r="D100" t="str">
+      <c r="D106" t="str">
         <v>Note Input All input field</v>
       </c>
-      <c r="E100" t="str">
+      <c r="E106" t="str">
         <v>[data-testid="location-settings-section-notes"] textarea</v>
       </c>
-      <c r="F100" t="str" xml:space="preserve">
+      <c r="F106" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
 2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
 3. Open the Notes tab.
 4. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
       </c>
-      <c r="G100" t="str">
+      <c r="G106" t="str">
         <v>Child</v>
       </c>
-      <c r="H100" t="str">
+      <c r="H106" t="str">
         <v>Child element only — the container "location-settings-section-notes" already has a data-testid; add one to the element inside it.</v>
       </c>
-      <c r="I100" t="str">
+      <c r="I106" t="str">
         <v>LOW</v>
       </c>
-      <c r="J100" t="str">
+      <c r="J106" t="str">
         <v>location-settings-input-note-input-all</v>
       </c>
-      <c r="K100" t="str">
+      <c r="K106" t="str">
         <v>location-settings-section-notes</v>
       </c>
-      <c r="L100" t="str">
+      <c r="L106" t="str">
         <v>[data-testid="location-settings-section-notes"] textarea</v>
       </c>
-      <c r="M100" t="str">
-        <v/>
-      </c>
-      <c r="N100" t="str">
+      <c r="M106" t="str">
+        <v/>
+      </c>
+      <c r="N106" t="str">
         <v>$$('[data-testid="location-settings-section-notes"] textarea')</v>
       </c>
-      <c r="O100" t="str">
-        <v/>
-      </c>
-      <c r="P100" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="101" xml:space="preserve">
-      <c r="A101" t="str">
+      <c r="O106" t="str">
+        <v/>
+      </c>
+      <c r="P106" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="107" xml:space="preserve">
+      <c r="A107" t="str">
         <v>NOT-006</v>
       </c>
-      <c r="B101" t="str">
-        <v>Location Settings</v>
-      </c>
-      <c r="C101" t="str">
+      <c r="B107" t="str">
+        <v>Location Settings</v>
+      </c>
+      <c r="C107" t="str">
         <v>Notes</v>
       </c>
-      <c r="D101" t="str">
+      <c r="D107" t="str">
         <v>Notes Delete button</v>
       </c>
-      <c r="E101" t="str">
+      <c r="E107" t="str">
         <v>[data-testid="location-settings-section-notes"] button:has-text("Delete")</v>
       </c>
-      <c r="F101" t="str" xml:space="preserve">
+      <c r="F107" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
 2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
 3. Open the Notes tab.
 4. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
       </c>
-      <c r="G101" t="str">
+      <c r="G107" t="str">
         <v>Child</v>
       </c>
-      <c r="H101" t="str">
+      <c r="H107" t="str">
         <v>Child element only — the container "location-settings-section-notes" already has a data-testid; add one to the element inside it.</v>
       </c>
-      <c r="I101" t="str">
+      <c r="I107" t="str">
         <v>LOW</v>
       </c>
-      <c r="J101" t="str">
+      <c r="J107" t="str">
         <v>location-settings-btn-notes-delete</v>
       </c>
-      <c r="K101" t="str">
+      <c r="K107" t="str">
         <v>location-settings-section-notes</v>
       </c>
-      <c r="L101" t="str">
+      <c r="L107" t="str">
         <v>[data-testid="location-settings-section-notes"] button</v>
       </c>
-      <c r="M101" t="str">
+      <c r="M107" t="str">
         <v>Delete</v>
       </c>
-      <c r="N101" t="str">
+      <c r="N107" t="str">
         <v>$$('[data-testid="location-settings-section-notes"] button').filter(e =&gt; (e.innerText || e.getAttribute('aria-label') || e.placeholder || '').includes('Delete'))</v>
       </c>
-      <c r="O101" t="str">
-        <v/>
-      </c>
-      <c r="P101" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="102" xml:space="preserve">
-      <c r="A102" t="str">
+      <c r="O107" t="str">
+        <v/>
+      </c>
+      <c r="P107" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="108" xml:space="preserve">
+      <c r="A108" t="str">
         <v>PRI-013</v>
       </c>
-      <c r="B102" t="str">
-        <v>Location Settings</v>
-      </c>
-      <c r="C102" t="str">
+      <c r="B108" t="str">
+        <v>Location Settings</v>
+      </c>
+      <c r="C108" t="str">
         <v>Pricing</v>
       </c>
-      <c r="D102" t="str">
+      <c r="D108" t="str">
         <v>Stay button</v>
       </c>
-      <c r="E102" t="str">
+      <c r="E108" t="str">
         <v>[data-testid="location-settings-modal-unsaved-changes"] button:has-text("Stay")</v>
       </c>
-      <c r="F102" t="str" xml:space="preserve">
+      <c r="F108" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
 2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
 3. Open the Pricing tab.
 4. Change any field, then navigate away without saving (for example click Home in the sidebar). (opens the unsaved changes dialog)
 5. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
       </c>
-      <c r="G102" t="str">
+      <c r="G108" t="str">
         <v>Child</v>
       </c>
-      <c r="H102" t="str">
+      <c r="H108" t="str">
         <v>Child element only — the container "location-settings-modal-unsaved-changes" already has a data-testid; add one to the element inside it.</v>
       </c>
-      <c r="I102" t="str">
+      <c r="I108" t="str">
         <v>LOW</v>
       </c>
-      <c r="J102" t="str">
+      <c r="J108" t="str">
         <v>location-settings-btn-stay</v>
       </c>
-      <c r="K102" t="str">
+      <c r="K108" t="str">
         <v>location-settings-modal-unsaved-changes</v>
       </c>
-      <c r="L102" t="str">
+      <c r="L108" t="str">
         <v>[data-testid="location-settings-modal-unsaved-changes"] button</v>
       </c>
-      <c r="M102" t="str">
+      <c r="M108" t="str">
         <v>Stay</v>
       </c>
-      <c r="N102" t="str">
+      <c r="N108" t="str">
         <v>$$('[data-testid="location-settings-modal-unsaved-changes"] button').filter(e =&gt; (e.innerText || e.getAttribute('aria-label') || e.placeholder || '').includes('Stay'))</v>
       </c>
-      <c r="O102" t="str">
-        <v/>
-      </c>
-      <c r="P102" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="103" xml:space="preserve">
-      <c r="A103" t="str">
-        <v>DLG-007</v>
-      </c>
-      <c r="B103" t="str">
-        <v>Location Settings</v>
-      </c>
-      <c r="C103" t="str">
+      <c r="O108" t="str">
+        <v/>
+      </c>
+      <c r="P108" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="109" xml:space="preserve">
+      <c r="A109" t="str">
+        <v>DLG-009</v>
+      </c>
+      <c r="B109" t="str">
+        <v>Location Settings</v>
+      </c>
+      <c r="C109" t="str">
         <v>Shared dialogs (all tabs)</v>
       </c>
-      <c r="D103" t="str">
+      <c r="D109" t="str">
         <v>Unsaved Changes Ok button</v>
       </c>
-      <c r="E103" t="str">
+      <c r="E109" t="str">
         <v>[data-testid="location-settings-modal-unsaved-changes"] button:has-text("Discard")</v>
       </c>
-      <c r="F103" t="str" xml:space="preserve">
+      <c r="F109" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
 2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
 3. Open any tab — this surface is shared by all of them.
 4. Change any field, then navigate away without saving (for example click Home in the sidebar). (opens the unsaved changes dialog)
 5. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
       </c>
-      <c r="G103" t="str">
+      <c r="G109" t="str">
         <v>Child</v>
       </c>
-      <c r="H103" t="str">
+      <c r="H109" t="str">
         <v>Child element only — the container "location-settings-modal-unsaved-changes" already has a data-testid; add one to the element inside it.</v>
       </c>
-      <c r="I103" t="str">
+      <c r="I109" t="str">
         <v>LOW</v>
       </c>
-      <c r="J103" t="str">
+      <c r="J109" t="str">
         <v>location-settings-btn-unsaved-changes-ok</v>
       </c>
-      <c r="K103" t="str">
+      <c r="K109" t="str">
         <v>location-settings-modal-unsaved-changes</v>
       </c>
-      <c r="L103" t="str">
+      <c r="L109" t="str">
         <v>[data-testid="location-settings-modal-unsaved-changes"] button</v>
       </c>
-      <c r="M103" t="str">
+      <c r="M109" t="str">
         <v>Discard</v>
       </c>
-      <c r="N103" t="str">
+      <c r="N109" t="str">
         <v>$$('[data-testid="location-settings-modal-unsaved-changes"] button').filter(e =&gt; (e.innerText || e.getAttribute('aria-label') || e.placeholder || '').includes('Discard'))</v>
       </c>
-      <c r="O103" t="str">
-        <v/>
-      </c>
-      <c r="P103" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="104" xml:space="preserve">
-      <c r="A104" t="str">
-        <v>DLG-008</v>
-      </c>
-      <c r="B104" t="str">
-        <v>Location Settings</v>
-      </c>
-      <c r="C104" t="str">
+      <c r="O109" t="str">
+        <v/>
+      </c>
+      <c r="P109" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="110" xml:space="preserve">
+      <c r="A110" t="str">
+        <v>DLG-010</v>
+      </c>
+      <c r="B110" t="str">
+        <v>Location Settings</v>
+      </c>
+      <c r="C110" t="str">
         <v>Shared dialogs (all tabs)</v>
       </c>
-      <c r="D104" t="str">
+      <c r="D110" t="str">
         <v>Unsaved Changes Cancel button</v>
       </c>
-      <c r="E104" t="str">
+      <c r="E110" t="str">
         <v>[data-testid="location-settings-modal-unsaved-changes"] button:has-text("Stay")</v>
       </c>
-      <c r="F104" t="str" xml:space="preserve">
+      <c r="F110" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
 2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
 3. Open any tab — this surface is shared by all of them.
 4. Change any field, then navigate away without saving (for example click Home in the sidebar). (opens the unsaved changes dialog)
 5. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
       </c>
-      <c r="G104" t="str">
+      <c r="G110" t="str">
         <v>Child</v>
       </c>
-      <c r="H104" t="str">
+      <c r="H110" t="str">
         <v>Child element only — the container "location-settings-modal-unsaved-changes" already has a data-testid; add one to the element inside it.</v>
       </c>
-      <c r="I104" t="str">
+      <c r="I110" t="str">
         <v>LOW</v>
       </c>
-      <c r="J104" t="str">
+      <c r="J110" t="str">
         <v>location-settings-btn-unsaved-changes-cancel</v>
       </c>
-      <c r="K104" t="str">
+      <c r="K110" t="str">
         <v>location-settings-modal-unsaved-changes</v>
       </c>
-      <c r="L104" t="str">
+      <c r="L110" t="str">
         <v>[data-testid="location-settings-modal-unsaved-changes"] button</v>
       </c>
-      <c r="M104" t="str">
+      <c r="M110" t="str">
         <v>Stay</v>
       </c>
-      <c r="N104" t="str">
+      <c r="N110" t="str">
         <v>$$('[data-testid="location-settings-modal-unsaved-changes"] button').filter(e =&gt; (e.innerText || e.getAttribute('aria-label') || e.placeholder || '').includes('Stay'))</v>
       </c>
-      <c r="O104" t="str">
-        <v/>
-      </c>
-      <c r="P104" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="105" xml:space="preserve">
-      <c r="A105" t="str">
+      <c r="O110" t="str">
+        <v/>
+      </c>
+      <c r="P110" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="111" xml:space="preserve">
+      <c r="A111" t="str">
         <v>SSL-007</v>
       </c>
-      <c r="B105" t="str">
-        <v>Location Settings</v>
-      </c>
-      <c r="C105" t="str">
+      <c r="B111" t="str">
+        <v>Location Settings</v>
+      </c>
+      <c r="C111" t="str">
         <v>Shared Setup Locations</v>
       </c>
-      <c r="D105" t="str">
+      <c r="D111" t="str">
         <v>Change Local Office Heading dialog</v>
       </c>
-      <c r="E105" t="str">
+      <c r="E111" t="str">
         <v>[data-testid="location-settings-modal-change-local-office"] h2</v>
       </c>
-      <c r="F105" t="str" xml:space="preserve">
+      <c r="F111" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
 2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
 3. Open the Shared Setup Locations tab.
 4. Click the Add button in the last row of the Shared Setup Locations grid. (opens the change local office dialog)
 5. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
       </c>
-      <c r="G105" t="str">
+      <c r="G111" t="str">
         <v>Child</v>
       </c>
-      <c r="H105" t="str">
+      <c r="H111" t="str">
         <v>Child element only — the container "location-settings-modal-change-local-office" already has a data-testid; add one to the element inside it.</v>
       </c>
-      <c r="I105" t="str">
+      <c r="I111" t="str">
         <v>LOW</v>
       </c>
-      <c r="J105" t="str">
+      <c r="J111" t="str">
         <v>location-settings-modal-change-local-office-heading</v>
       </c>
-      <c r="K105" t="str">
+      <c r="K111" t="str">
         <v>location-settings-modal-change-local-office</v>
       </c>
-      <c r="L105" t="str">
+      <c r="L111" t="str">
         <v>[data-testid="location-settings-modal-change-local-office"] h2</v>
       </c>
-      <c r="M105" t="str">
-        <v/>
-      </c>
-      <c r="N105" t="str">
+      <c r="M111" t="str">
+        <v/>
+      </c>
+      <c r="N111" t="str">
         <v>$$('[data-testid="location-settings-modal-change-local-office"] h2')</v>
       </c>
-      <c r="O105" t="str">
-        <v/>
-      </c>
-      <c r="P105" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="106" xml:space="preserve">
-      <c r="A106" t="str">
+      <c r="O111" t="str">
+        <v/>
+      </c>
+      <c r="P111" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="112" xml:space="preserve">
+      <c r="A112" t="str">
         <v>SSL-008</v>
       </c>
-      <c r="B106" t="str">
-        <v>Location Settings</v>
-      </c>
-      <c r="C106" t="str">
+      <c r="B112" t="str">
+        <v>Location Settings</v>
+      </c>
+      <c r="C112" t="str">
         <v>Shared Setup Locations</v>
       </c>
-      <c r="D106" t="str">
+      <c r="D112" t="str">
         <v>Dlg Results table</v>
       </c>
-      <c r="E106" t="str">
+      <c r="E112" t="str">
         <v>[data-testid="location-settings-modal-change-local-office"] table</v>
       </c>
-      <c r="F106" t="str" xml:space="preserve">
+      <c r="F112" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
 2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
 3. Open the Shared Setup Locations tab.
 4. Click the Add button in the last row of the Shared Setup Locations grid. (opens the change local office dialog)
 5. Press F12, open Elements, press Ctrl+F and paste the selector from the "Current selector" column.</v>
       </c>
-      <c r="G106" t="str">
+      <c r="G112" t="str">
         <v>Child</v>
       </c>
-      <c r="H106" t="str">
+      <c r="H112" t="str">
         <v>Child element only — the container "location-settings-modal-change-local-office" already has a data-testid; add one to the element inside it.</v>
       </c>
-      <c r="I106" t="str">
+      <c r="I112" t="str">
         <v>LOW</v>
       </c>
-      <c r="J106" t="str">
+      <c r="J112" t="str">
         <v>location-settings-table-dlg-results</v>
       </c>
-      <c r="K106" t="str">
+      <c r="K112" t="str">
         <v>location-settings-modal-change-local-office</v>
       </c>
-      <c r="L106" t="str">
+      <c r="L112" t="str">
         <v>[data-testid="location-settings-modal-change-local-office"] table</v>
       </c>
-      <c r="M106" t="str">
-        <v/>
-      </c>
-      <c r="N106" t="str">
+      <c r="M112" t="str">
+        <v/>
+      </c>
+      <c r="N112" t="str">
         <v>$$('[data-testid="location-settings-modal-change-local-office"] table')</v>
       </c>
-      <c r="O106" t="str">
-        <v/>
-      </c>
-      <c r="P106" t="str">
+      <c r="O112" t="str">
+        <v/>
+      </c>
+      <c r="P112" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P106"/>
+  <autoFilter ref="A1:P112"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P106"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P112"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F47"/>
   <cols>
     <col min="1" max="1" width="60.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -7528,7 +7847,7 @@
         <v>Setup &gt; Location Settings &gt; Location Management History</v>
       </c>
       <c r="B40" t="str">
-        <v>HIS-006, HIS-007, HIS-008, HIS-009, HIS-010, HIS-003, HIS-004, HIS-005</v>
+        <v>HIS-014, HIS-007, HIS-008, HIS-009, HIS-010, HIS-011, HIS-012, HIS-003, HIS-004, HIS-005, HIS-006, HIS-013</v>
       </c>
       <c r="C40" t="str">
         <v>MEDIUM</v>
@@ -7540,10 +7859,10 @@
 4. Press F12, open Elements, press Ctrl+F and paste the selector below.</v>
       </c>
       <c r="E40" t="str">
-        <v>[data-testid="location-settings-tab-content-management-history"] button[role="combobox"]:not([data-testid="location-settings-select-history-type"])</v>
+        <v>[data-testid="location-settings-tab-content-management-history"] table[data-slot="table"]</v>
       </c>
       <c r="F40" t="str">
-        <v/>
+        <v>Delete</v>
       </c>
     </row>
     <row r="41" xml:space="preserve">
@@ -7571,103 +7890,150 @@
     </row>
     <row r="42" xml:space="preserve">
       <c r="A42" t="str">
+        <v>Setup &gt; Location Settings &gt; any tab</v>
+      </c>
+      <c r="B42" t="str">
+        <v>DLG-007</v>
+      </c>
+      <c r="C42" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="D42" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Sign in to Navigator Cloud.
+2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
+3. Open any tab — this surface is shared by all of them.
+4. Press F12, open Elements, press Ctrl+F and paste the selector below.</v>
+      </c>
+      <c r="E42" t="str">
+        <v>[data-sidebar="footer"] button[data-slot="dropdown-menu-trigger"]</v>
+      </c>
+      <c r="F42" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="43" xml:space="preserve">
+      <c r="A43" t="str">
+        <v>Setup &gt; Location Settings &gt; any tab &gt; open the column menu</v>
+      </c>
+      <c r="B43" t="str">
+        <v>DLG-008</v>
+      </c>
+      <c r="C43" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="D43" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Sign in to Navigator Cloud.
+2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
+3. Open any tab — this surface is shared by all of them.
+4. Click a column header, then open its menu.
+5. Press F12, open Elements, press Ctrl+F and paste the selector below.</v>
+      </c>
+      <c r="E43" t="str">
+        <v>[role="menu"] [role="menuitem"][aria-haspopup="menu"]</v>
+      </c>
+      <c r="F43" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="44" xml:space="preserve">
+      <c r="A44" t="str">
         <v>Setup &gt; Location Settings &gt; Account and Address &gt; open the "account list" dialog</v>
       </c>
-      <c r="B42" t="str">
+      <c r="B44" t="str">
         <v>AA-020, AA-021, AA-019</v>
       </c>
-      <c r="C42" t="str">
+      <c r="C44" t="str">
         <v>LOW</v>
       </c>
-      <c r="D42" t="str" xml:space="preserve">
+      <c r="D44" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
 2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
 3. Open the Account and Address tab.
 4. Click the lookup button beside the Venue/Branch Account name. (opens the account list dialog)
 5. Press F12, open Elements, press Ctrl+F and paste the selector below.</v>
       </c>
-      <c r="E42" t="str">
+      <c r="E44" t="str">
         <v>[data-testid="location-settings-modal-account-list"] button</v>
       </c>
-      <c r="F42" t="str">
+      <c r="F44" t="str">
         <v>Close</v>
       </c>
     </row>
-    <row r="43" xml:space="preserve">
-      <c r="A43" t="str">
+    <row r="45" xml:space="preserve">
+      <c r="A45" t="str">
         <v>Setup &gt; Location Settings &gt; any tab &gt; open the "unsaved changes" dialog</v>
       </c>
-      <c r="B43" t="str">
-        <v>DLG-007, DLG-008</v>
-      </c>
-      <c r="C43" t="str">
+      <c r="B45" t="str">
+        <v>DLG-009, DLG-010</v>
+      </c>
+      <c r="C45" t="str">
         <v>LOW</v>
       </c>
-      <c r="D43" t="str" xml:space="preserve">
+      <c r="D45" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
 2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
 3. Open any tab — this surface is shared by all of them.
 4. Change any field, then navigate away without saving (for example click Home in the sidebar). (opens the unsaved changes dialog)
 5. Press F12, open Elements, press Ctrl+F and paste the selector below.</v>
       </c>
-      <c r="E43" t="str">
+      <c r="E45" t="str">
         <v>[data-testid="location-settings-modal-unsaved-changes"] button</v>
       </c>
-      <c r="F43" t="str">
+      <c r="F45" t="str">
         <v>Discard | Stay</v>
       </c>
     </row>
-    <row r="44" xml:space="preserve">
-      <c r="A44" t="str">
+    <row r="46" xml:space="preserve">
+      <c r="A46" t="str">
         <v>Setup &gt; Location Settings &gt; Auto Add-On &gt; open the "unsaved changes" dialog</v>
       </c>
-      <c r="B44" t="str">
+      <c r="B46" t="str">
         <v>AAO-006</v>
       </c>
-      <c r="C44" t="str">
+      <c r="C46" t="str">
         <v>LOW</v>
       </c>
-      <c r="D44" t="str" xml:space="preserve">
+      <c r="D46" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
 2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
 3. Open the Auto Add-On tab.
 4. Change any field, then navigate away without saving (for example click Home in the sidebar). (opens the unsaved changes dialog)
 5. Press F12, open Elements, press Ctrl+F and paste the selector below.</v>
       </c>
-      <c r="E44" t="str">
+      <c r="E46" t="str">
         <v>[data-testid="location-settings-modal-unsaved-changes"] h2</v>
       </c>
-      <c r="F44" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="45" xml:space="preserve">
-      <c r="A45" t="str">
+      <c r="F46" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="47" xml:space="preserve">
+      <c r="A47" t="str">
         <v>Setup &gt; Location Settings &gt; Pricing &gt; open the "unsaved changes" dialog</v>
       </c>
-      <c r="B45" t="str">
+      <c r="B47" t="str">
         <v>PRI-013</v>
       </c>
-      <c r="C45" t="str">
+      <c r="C47" t="str">
         <v>LOW</v>
       </c>
-      <c r="D45" t="str" xml:space="preserve">
+      <c r="D47" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in to Navigator Cloud.
 2. Go to Setup &gt; Location Settings and open office 1604 — the office the suite runs against.
 3. Open the Pricing tab.
 4. Change any field, then navigate away without saving (for example click Home in the sidebar). (opens the unsaved changes dialog)
 5. Press F12, open Elements, press Ctrl+F and paste the selector below.</v>
       </c>
-      <c r="E45" t="str">
+      <c r="E47" t="str">
         <v>[data-testid="location-settings-modal-unsaved-changes"] button</v>
       </c>
-      <c r="F45" t="str">
+      <c r="F47" t="str">
         <v>Stay</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F45"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F47"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>